<commit_message>
updated wordcloud python script
output frequencies to excel
</commit_message>
<xml_diff>
--- a/do/learn/subwords.xlsx
+++ b/do/learn/subwords.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christinasun/Library/CloudStorage/Dropbox/Davis/Research_Projects/Ed Lab GSR/csac/do/learn/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3F6C50AA-28A4-FC40-B79B-667C60FCD9C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6486B9D-9656-7447-8063-579473605865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3080" yWindow="2060" windowWidth="28040" windowHeight="17440" xr2:uid="{A66D55BB-4903-8B4A-B41D-B2EC86BA5ABB}"/>
   </bookViews>
@@ -36,12 +36,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
-  <si>
-    <t>NON CONFORMING</t>
-  </si>
-  <si>
-    <t>NONCONFORMING</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>non conforming</t>
+  </si>
+  <si>
+    <t>nonconforming</t>
+  </si>
+  <si>
+    <t>quee5</t>
+  </si>
+  <si>
+    <t>queer</t>
+  </si>
+  <si>
+    <t>gender fluid</t>
+  </si>
+  <si>
+    <t>genderfluid</t>
   </si>
 </sst>
 </file>
@@ -393,7 +405,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A07A1D28-E9EB-744B-AFCA-10F24204A46B}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -404,6 +416,22 @@
         <v>1</v>
       </c>
     </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>